<commit_message>
Add product catalog test cases and enhancement requests
</commit_message>
<xml_diff>
--- a/docs/BugReports/Bug_Reports.xlsx
+++ b/docs/BugReports/Bug_Reports.xlsx
@@ -450,7 +450,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -523,16 +523,11 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -611,11 +606,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -660,7 +659,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -669,15 +668,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -757,15 +756,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>222480</xdr:colOff>
+      <xdr:colOff>238680</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>900720</xdr:rowOff>
+      <xdr:rowOff>1009800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>2180520</xdr:colOff>
+      <xdr:colOff>2196360</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>1700280</xdr:rowOff>
+      <xdr:rowOff>1809000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -778,8 +777,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10530360" y="7625880"/>
-          <a:ext cx="1958040" cy="799560"/>
+          <a:off x="10546560" y="6610680"/>
+          <a:ext cx="1957680" cy="799200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -795,15 +794,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>475920</xdr:colOff>
+      <xdr:colOff>443520</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>785520</xdr:rowOff>
+      <xdr:rowOff>998640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1938600</xdr:colOff>
+      <xdr:colOff>1905840</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>1280160</xdr:rowOff>
+      <xdr:rowOff>1492920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -816,8 +815,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10783800" y="5715000"/>
-          <a:ext cx="1462680" cy="494640"/>
+          <a:off x="10751400" y="4803480"/>
+          <a:ext cx="1462320" cy="494280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -944,338 +943,354 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="34.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="34.48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="95.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+    <row r="2" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="2"/>
+      <c r="N2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="184.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="5" t="s">
+    <row r="3" customFormat="false" ht="163.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
+      <c r="L3" s="8"/>
+      <c r="M3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="2"/>
+      <c r="N3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="5" t="s">
+    <row r="4" customFormat="false" ht="76.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3"/>
+      <c r="B4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="11" t="s">
+      <c r="L4" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="2"/>
+      <c r="N4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="141.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="3"/>
+      <c r="B5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="K5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="L5" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="N5" s="2"/>
+      <c r="N5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="3"/>
+      <c r="B6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="L6" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="N6" s="2"/>
+      <c r="N6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="5" t="s">
+    <row r="7" customFormat="false" ht="65.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3"/>
+      <c r="B7" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="2"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="3"/>
+      <c r="B8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="5"/>
+      <c r="C8" s="6"/>
       <c r="D8" s="16"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="2"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="3"/>
+      <c r="B9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="2"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="3"/>
+      <c r="B10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="2"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="3"/>
+      <c r="B11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="2"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="3"/>
+      <c r="B12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="2"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add checkout test cases and validation bug reports
</commit_message>
<xml_diff>
--- a/docs/BugReports/Bug_Reports.xlsx
+++ b/docs/BugReports/Bug_Reports.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="99">
   <si>
     <t xml:space="preserve">Bug Report</t>
   </si>
@@ -31,6 +31,9 @@
     <t xml:space="preserve">Module </t>
   </si>
   <si>
+    <t xml:space="preserve">TC_ID</t>
+  </si>
+  <si>
     <t xml:space="preserve">Title </t>
   </si>
   <si>
@@ -43,9 +46,6 @@
     <t xml:space="preserve">Actual Result</t>
   </si>
   <si>
-    <t xml:space="preserve">TC_ID</t>
-  </si>
-  <si>
     <t xml:space="preserve">Priority </t>
   </si>
   <si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">Registration </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg-08</t>
   </si>
   <si>
     <t xml:space="preserve">Registration form accepts whitespace-only input and returns misleading error message</t>
@@ -168,9 +171,6 @@
     <t xml:space="preserve">User receives a „This user already exists“ pop-up</t>
   </si>
   <si>
-    <t xml:space="preserve">Reg-08</t>
-  </si>
-  <si>
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
@@ -189,6 +189,9 @@
     <t xml:space="preserve">Login</t>
   </si>
   <si>
+    <t xml:space="preserve">Log-05</t>
+  </si>
+  <si>
     <t xml:space="preserve">Attempted login with wrong credentials gives specific info</t>
   </si>
   <si>
@@ -287,9 +290,6 @@
     <t xml:space="preserve">User receives a „Wrong password.“ pop-up</t>
   </si>
   <si>
-    <t xml:space="preserve">Log-05</t>
-  </si>
-  <si>
     <t xml:space="preserve">High</t>
   </si>
   <si>
@@ -299,6 +299,9 @@
     <t xml:space="preserve">B_003</t>
   </si>
   <si>
+    <t xml:space="preserve">Log-08</t>
+  </si>
+  <si>
     <t xml:space="preserve">Authentication allows login using whitespace-only credentials</t>
   </si>
   <si>
@@ -392,9 +395,6 @@
   </si>
   <si>
     <t xml:space="preserve">The application accepts whitespace-only credentials and grants an authenticated session. The navigation bar changes to a logged-in state and displays "Welcome" without requiring valid credentials. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Log-08</t>
   </si>
   <si>
     <t xml:space="preserve">Critical</t>
@@ -407,6 +407,9 @@
     <t xml:space="preserve">B_004</t>
   </si>
   <si>
+    <t xml:space="preserve">Log-09</t>
+  </si>
+  <si>
     <t xml:space="preserve">Authentication allows login with script tag input as credentials</t>
   </si>
   <si>
@@ -417,9 +420,6 @@
     <t xml:space="preserve">User is logged in after entering &lt;script&gt;alert('test')&lt;/script&gt; as credentials. The system displays the script string as the logged-in username.</t>
   </si>
   <si>
-    <t xml:space="preserve">Log-09</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 Risk: Possible authentication bypass and stored XSS/user input sanitization issue.</t>
   </si>
@@ -427,19 +427,822 @@
     <t xml:space="preserve">B_005</t>
   </si>
   <si>
+    <t xml:space="preserve">Cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CART-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Products added to cart are not carried over after login.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click on a product</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">  
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click add to car</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">t 
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Login</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 
+ 4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click on cart</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">The chosen product is added to cart and visible after login.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The product in not transferred to the cart after login.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It would mostly affect first time users of the website that add their desired products to cart before creating an account.</t>
+  </si>
+  <si>
     <t xml:space="preserve">B_006</t>
   </si>
   <si>
+    <t xml:space="preserve">Checkout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORD-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with empty cart</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User is displayed an error message or a pop-up stating that the cart is currently empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A success message “Thank you for your purchase!” appears</t>
+  </si>
+  <si>
     <t xml:space="preserve">B_007</t>
   </si>
   <si>
+    <t xml:space="preserve">ORD-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with empty Country field</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials leaving Country field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User is displayed an error message or a pop-up stating that all fields need to be filled to complete purchase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order is successfully placed and confirmation message is displayed.
+User is provided with Order ID.</t>
+  </si>
+  <si>
     <t xml:space="preserve">B_008</t>
   </si>
   <si>
+    <t xml:space="preserve">ORD-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with empty City field</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials leaving City field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">B_009</t>
   </si>
   <si>
+    <t xml:space="preserve">ORD-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with empty Month field</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials leaving Month field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">B_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORD-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with empty Year field</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials leaving Year field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">B_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORD-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with invalid Credit Card number format</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out Credit Card field with letters
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill the rest of the fields with valid credentials
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User is displayed an error message or a pop-up stating that one or more fields have invalid data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORD-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users are provided with Order ID when completing purchase with expired card data</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with provided dummy credentials
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">B_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORD-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Place order with very long input values</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Copy and paste each data 3 times in the provided field
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Order is successfully placed and confirmation message is displayed. User is provided with Order ID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORD-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Success confirmation modal does not block interaction with underlying page</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on Place order button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fill out form with valid dummy credentials
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Click on purchase
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">4. DO NOT CLOSE CONFIRMATION WINDOW
+5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Click on purchase</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User is not able to interact with the background or other fields until confirmation pop-up message is closed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is able to put multiple orders and is provided new and different Order ID every time.</t>
   </si>
 </sst>
 </file>
@@ -450,7 +1253,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -529,6 +1332,19 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -606,7 +1422,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -659,19 +1475,23 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -762,9 +1582,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>2196360</xdr:colOff>
+      <xdr:colOff>2196000</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>1809000</xdr:rowOff>
+      <xdr:rowOff>1808640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -777,8 +1597,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10546560" y="6610680"/>
-          <a:ext cx="1957680" cy="799200"/>
+          <a:off x="11551320" y="7048800"/>
+          <a:ext cx="1957320" cy="798840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -800,9 +1620,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1905840</xdr:colOff>
+      <xdr:colOff>1905480</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>1492920</xdr:rowOff>
+      <xdr:rowOff>1492560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -815,8 +1635,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10751400" y="4803480"/>
-          <a:ext cx="1462320" cy="494280"/>
+          <a:off x="11756160" y="5132520"/>
+          <a:ext cx="1461960" cy="493920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -943,12 +1763,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="34.48"/>
   </cols>
   <sheetData>
@@ -978,10 +1799,10 @@
       <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F2" s="4" t="s">
@@ -1010,7 +1831,7 @@
       </c>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="163.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="184.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="6" t="s">
         <v>13</v>
@@ -1021,10 +1842,10 @@
       <c r="D3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="6" t="s">
@@ -1048,7 +1869,7 @@
       </c>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="76.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3"/>
       <c r="B4" s="6" t="s">
         <v>24</v>
@@ -1056,13 +1877,13 @@
       <c r="C4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>28</v>
       </c>
       <c r="G4" s="10" t="s">
@@ -1088,7 +1909,7 @@
       </c>
       <c r="N4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="141.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="150" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3"/>
       <c r="B5" s="6" t="s">
         <v>33</v>
@@ -1096,17 +1917,17 @@
       <c r="C5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="13" t="s">
+      <c r="F5" s="11" t="s">
         <v>36</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>18</v>
       </c>
       <c r="H5" s="14" t="s">
         <v>37</v>
@@ -1136,19 +1957,19 @@
       <c r="C6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="10" t="s">
+      <c r="E6" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="F6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="6" t="s">
         <v>44</v>
       </c>
       <c r="I6" s="6" t="s">
@@ -1168,152 +1989,386 @@
       </c>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="65.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
+      <c r="C7" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
       <c r="B8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
+        <v>54</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="138.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3"/>
       <c r="B9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
+        <v>61</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="127.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
       <c r="B10" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
+        <v>67</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="L10" s="6"/>
       <c r="M10" s="6"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="130.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
       <c r="B11" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
+        <v>71</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="119.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
       <c r="B12" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
+        <v>75</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="L12" s="6"/>
       <c r="M12" s="6"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
+    <row r="13" customFormat="false" ht="141.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18"/>
+      <c r="B13" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="18"/>
+    </row>
+    <row r="14" customFormat="false" ht="109.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+    </row>
+    <row r="15" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I3:I12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I3:I16" type="list">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K3:K12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K3:K16" type="list">
       <formula1>"Always,Often,Rare,Never,"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="L3:L5 L7:L12" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="L3:L5 L7:L16" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M3:M12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M3:M16" type="list">
       <formula1>"Open,In Review,Assigned,Not Relevant,Repeated"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J3:J12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J3:J16" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Complete About Us module and add manual testing summary
</commit_message>
<xml_diff>
--- a/docs/BugReports/Bug_Reports.xlsx
+++ b/docs/BugReports/Bug_Reports.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="114">
   <si>
     <t xml:space="preserve">Bug Report</t>
   </si>
@@ -545,6 +545,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -554,6 +555,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -565,6 +567,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -574,6 +577,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials
 </t>
@@ -585,6 +589,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -594,6 +599,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -621,6 +627,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -630,6 +637,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -641,6 +649,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -650,6 +659,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials leaving Country field empty
 </t>
@@ -661,6 +671,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -670,6 +681,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -698,6 +710,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -707,6 +720,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -718,6 +732,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -727,6 +742,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials leaving City field empty
 </t>
@@ -738,6 +754,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -747,6 +764,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -768,6 +786,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -777,6 +796,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -788,6 +808,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -797,6 +818,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials leaving Month field empty
 </t>
@@ -808,6 +830,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -817,6 +840,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -838,6 +862,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -847,6 +872,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -858,6 +884,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -867,6 +894,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials leaving Year field empty
 </t>
@@ -878,6 +906,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -887,6 +916,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -908,6 +938,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -917,6 +948,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -928,6 +960,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -937,6 +970,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out Credit Card field with letters
 </t>
@@ -948,6 +982,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3.</t>
     </r>
@@ -957,6 +992,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill the rest of the fields with valid credentials
 </t>
@@ -968,6 +1004,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">4. </t>
     </r>
@@ -977,6 +1014,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -1001,6 +1039,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -1010,6 +1049,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -1021,6 +1061,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -1030,6 +1071,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with provided dummy credentials
 </t>
@@ -1041,6 +1083,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -1050,6 +1093,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -1071,6 +1115,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -1080,6 +1125,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -1091,6 +1137,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -1100,6 +1147,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials
 </t>
@@ -1111,6 +1159,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3.</t>
     </r>
@@ -1120,6 +1169,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Copy and paste each data 3 times in the provided field
 </t>
@@ -1131,6 +1181,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">4. </t>
     </r>
@@ -1140,6 +1191,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase</t>
     </r>
@@ -1164,6 +1216,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1. </t>
     </r>
@@ -1173,6 +1226,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on Place order button
 </t>
@@ -1184,6 +1238,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.</t>
     </r>
@@ -1193,6 +1248,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Fill out form with valid dummy credentials
 </t>
@@ -1204,6 +1260,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3. </t>
     </r>
@@ -1213,6 +1270,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Click on purchase
 </t>
@@ -1224,6 +1282,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">4. DO NOT CLOSE CONFIRMATION WINDOW
 5.</t>
@@ -1234,6 +1293,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Click on purchase</t>
     </r>
@@ -1243,6 +1303,223 @@
   </si>
   <si>
     <t xml:space="preserve">User is able to put multiple orders and is provided new and different Order ID every time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONT-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact form allows message submission without required email address</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click on contact from nav-bar
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Input  data in the name and message fields
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Leave e-mail field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click on send message</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Error message or pop-up is displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User receives a pop-up stating : „Thanks for the message!!“</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONT-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact form allows message submission with invalid email address format</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click on contact from nav-bar
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Input  data in the name and message fields
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Type “abc” in e-mail field 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click on send message</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">B_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_020</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1530,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1332,19 +1609,6 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1422,7 +1686,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1485,18 +1749,6 @@
     </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1578,13 +1830,13 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>238680</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>1009800</xdr:rowOff>
+      <xdr:rowOff>925200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>2196000</xdr:colOff>
+      <xdr:colOff>2195280</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>1808640</xdr:rowOff>
+      <xdr:rowOff>1723320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1597,8 +1849,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11551320" y="7048800"/>
-          <a:ext cx="1957320" cy="798840"/>
+          <a:off x="11551320" y="5219640"/>
+          <a:ext cx="1956600" cy="798120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1614,15 +1866,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>443520</xdr:colOff>
+      <xdr:colOff>379440</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>998640</xdr:rowOff>
+      <xdr:rowOff>928080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1905480</xdr:colOff>
+      <xdr:colOff>1840680</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>1492560</xdr:rowOff>
+      <xdr:rowOff>1421280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1635,8 +1887,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11756160" y="5132520"/>
-          <a:ext cx="1461960" cy="493920"/>
+          <a:off x="11692080" y="3462840"/>
+          <a:ext cx="1461240" cy="493200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1763,11 +2015,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="34.48"/>
@@ -1831,7 +2083,7 @@
       </c>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="184.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="93.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="6" t="s">
         <v>13</v>
@@ -1869,7 +2121,7 @@
       </c>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3"/>
       <c r="B4" s="6" t="s">
         <v>24</v>
@@ -1909,7 +2161,7 @@
       </c>
       <c r="N4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="150" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="138.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3"/>
       <c r="B5" s="6" t="s">
         <v>33</v>
@@ -1989,7 +2241,7 @@
       </c>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
         <v>46</v>
@@ -2029,7 +2281,7 @@
       </c>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
       <c r="B8" s="6" t="s">
         <v>54</v>
@@ -2043,13 +2295,13 @@
       <c r="E8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I8" s="6" t="s">
@@ -2062,10 +2314,12 @@
         <v>22</v>
       </c>
       <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+      <c r="M8" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" customFormat="false" ht="138.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3"/>
       <c r="B9" s="6" t="s">
         <v>61</v>
@@ -2079,13 +2333,13 @@
       <c r="E9" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H9" s="17" t="s">
+      <c r="H9" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I9" s="6" t="s">
@@ -2098,10 +2352,12 @@
         <v>22</v>
       </c>
       <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
+      <c r="M9" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="127.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="69.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
       <c r="B10" s="6" t="s">
         <v>67</v>
@@ -2115,13 +2371,13 @@
       <c r="E10" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I10" s="6" t="s">
@@ -2134,10 +2390,12 @@
         <v>22</v>
       </c>
       <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
+      <c r="M10" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="130.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
       <c r="B11" s="6" t="s">
         <v>71</v>
@@ -2151,13 +2409,13 @@
       <c r="E11" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="G11" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I11" s="6" t="s">
@@ -2170,10 +2428,12 @@
         <v>22</v>
       </c>
       <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
+      <c r="M11" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="119.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="69.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
       <c r="B12" s="6" t="s">
         <v>75</v>
@@ -2187,13 +2447,13 @@
       <c r="E12" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="17" t="s">
+      <c r="G12" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I12" s="6" t="s">
@@ -2206,11 +2466,13 @@
         <v>22</v>
       </c>
       <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
+      <c r="M12" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="141.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18"/>
+    <row r="13" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3"/>
       <c r="B13" s="6" t="s">
         <v>79</v>
       </c>
@@ -2223,13 +2485,13 @@
       <c r="E13" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="H13" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I13" s="6" t="s">
@@ -2242,10 +2504,12 @@
         <v>22</v>
       </c>
       <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="18"/>
+      <c r="M13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="109.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="69.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
         <v>84</v>
       </c>
@@ -2258,13 +2522,13 @@
       <c r="E14" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="F14" s="16" t="s">
+      <c r="F14" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="H14" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I14" s="6" t="s">
@@ -2277,9 +2541,11 @@
         <v>22</v>
       </c>
       <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
+      <c r="M14" s="6" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="15" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
         <v>88</v>
       </c>
@@ -2292,10 +2558,10 @@
       <c r="E15" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="10" t="s">
         <v>83</v>
       </c>
       <c r="H15" s="6" t="s">
@@ -2311,7 +2577,9 @@
         <v>22</v>
       </c>
       <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
+      <c r="M15" s="6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
@@ -2326,13 +2594,13 @@
       <c r="E16" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="G16" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="H16" s="17" t="s">
+      <c r="H16" s="10" t="s">
         <v>98</v>
       </c>
       <c r="I16" s="6" t="s">
@@ -2345,30 +2613,176 @@
         <v>22</v>
       </c>
       <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
+      <c r="M16" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I3:I16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I3:I22" type="list">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K3:K16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K3:K22" type="list">
       <formula1>"Always,Often,Rare,Never,"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="L3:L5 L7:L16" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="L3:L5 L7:L22" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M3:M16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M3:M22" type="list">
       <formula1>"Open,In Review,Assigned,Not Relevant,Repeated"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J3:J16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J3:J22" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>